<commit_message>
feat(procurement): Supplier Pricing UI + harga PO (new_price) + supplier per-produk
- Supplier Pricing: halaman + tabel + modal Create/Update/View, kolom sesuai
  model (name/supplier/uom/price/status), subtitle sesuai judul. Tombol
  Import/Export + template supplier-pricing (header berstyle, contoh data);
  daftarkan ke IMPORTABLE_MODULES.
- Product: hapus field supplier_id (types + modal create/update/view).
- Purchase Order: input harga menulis ke `new_price` (price asal tetap);
  subtotal & total ikut terkalkulasi (sumItems pakai new_price). Supplier per
  baris wajib pilih produk dulu (disabled) & dicari dari supplier yang punya
  produk tsb (supplier-pricing). Validasi submit: tolak bila ada produk tanpa
  supplier. Ganti produk -> reset supplier.
- Purchase Request: sembunyikan kolom Price, Subtotal & Total di detail item.
- types/purchaseItem: field new_price + formItemToPayload kirim new_price
  (fallback ke price agar PR/GR/DO tidak memicu update harga).
</commit_message>
<xml_diff>
--- a/public/templates/chart-of-account.xlsx
+++ b/public/templates/chart-of-account.xlsx
@@ -49,7 +49,7 @@
       <color rgb="FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -63,6 +63,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF2563EB"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCCCCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCCCCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -101,12 +113,16 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -485,31 +501,31 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>1000</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>ASET</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>ASSET</v>
       </c>
-      <c r="D2" s="2" t="str">
+      <c r="D2" s="4" t="str">
         <v>DEBIT</v>
       </c>
-      <c r="E2" s="2" t="b">
+      <c r="E2" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="4" t="str">
         <v/>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="5">
         <v>1</v>
       </c>
-      <c r="H2" s="2" t="str">
+      <c r="H2" s="4" t="str">
         <v>Kelompok aset</v>
       </c>
-      <c r="I2" s="2" t="str">
+      <c r="I2" s="4" t="str">
         <v>01/08/2026 08:00</v>
       </c>
     </row>
@@ -532,7 +548,7 @@
       <c r="F3" s="2" t="str">
         <v>1000</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="6">
         <v>2</v>
       </c>
       <c r="H3" s="2" t="str">
@@ -543,31 +559,31 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="str">
+      <c r="A4" s="4" t="str">
         <v>1000.1200</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="4" t="str">
         <v>Piutang Usaha</v>
       </c>
-      <c r="C4" s="2" t="str">
+      <c r="C4" s="4" t="str">
         <v>ASSET</v>
       </c>
-      <c r="D4" s="2" t="str">
+      <c r="D4" s="4" t="str">
         <v>DEBIT</v>
       </c>
-      <c r="E4" s="2" t="b">
+      <c r="E4" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="F4" s="2" t="str">
+      <c r="F4" s="4" t="str">
         <v>1000</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="5">
         <v>2</v>
       </c>
-      <c r="H4" s="2" t="str">
+      <c r="H4" s="4" t="str">
         <v>Piutang pelanggan</v>
       </c>
-      <c r="I4" s="2" t="str">
+      <c r="I4" s="4" t="str">
         <v>01/08/2026 08:02</v>
       </c>
     </row>
@@ -590,7 +606,7 @@
       <c r="F5" s="2" t="str">
         <v/>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="6">
         <v>1</v>
       </c>
       <c r="H5" s="2" t="str">
@@ -601,31 +617,31 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="str">
+      <c r="A6" s="4" t="str">
         <v>4000.4100</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B6" s="4" t="str">
         <v>Pendapatan Penjualan</v>
       </c>
-      <c r="C6" s="2" t="str">
+      <c r="C6" s="4" t="str">
         <v>REVENUE</v>
       </c>
-      <c r="D6" s="2" t="str">
+      <c r="D6" s="4" t="str">
         <v>CREDIT</v>
       </c>
-      <c r="E6" s="2" t="b">
+      <c r="E6" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="F6" s="2" t="str">
+      <c r="F6" s="4" t="str">
         <v>4000</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="5">
         <v>2</v>
       </c>
-      <c r="H6" s="2" t="str">
+      <c r="H6" s="4" t="str">
         <v>Penjualan barang</v>
       </c>
-      <c r="I6" s="2" t="str">
+      <c r="I6" s="4" t="str">
         <v>01/08/2026 08:04</v>
       </c>
     </row>

</xml_diff>